<commit_message>
Se completa [TC-003] Registro fallido por contraseñas no coincidentes
</commit_message>
<xml_diff>
--- a/testData/TutorialsNinja_RegisterPage.xlsx
+++ b/testData/TutorialsNinja_RegisterPage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erickfloresovando/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38FBCD51-B018-E046-AD62-6460FFECBE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{026B1D3B-46F3-A246-933A-B9A56E05261B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15600" xr2:uid="{A4E39AE2-BE39-2E44-9441-96961B052630}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="27">
   <si>
     <t>First Name</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>0OAu0u?M!Kj^Ex&lt;2i</t>
+  </si>
+  <si>
+    <t>$a}n5:vJ&lt;k!CRgL</t>
   </si>
 </sst>
 </file>
@@ -549,27 +552,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="6">
-        <v>5551234567</v>
+        <v>5554443322</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{5C5E8BDF-807F-974A-926D-5FE93B49A08D}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{21DBB730-C1B9-314F-A6B9-95E74C29DB84}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -577,7 +580,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B37700-12D2-C148-BC78-07B523A0C6B2}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15.1640625" bestFit="1" customWidth="1"/>
@@ -647,52 +650,73 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="6">
+        <v>5551234567</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D11" s="6">
         <v>5554443322</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D12" s="6">
         <v>5527456798</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>25</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{2994E8E3-27A4-3342-A375-5CF20C5E6751}"/>
-    <hyperlink ref="C5" r:id="rId2" xr:uid="{2ED25ACD-8A16-DD42-8FB2-9069856DDED4}"/>
-    <hyperlink ref="C6" r:id="rId3" xr:uid="{432655B1-7C28-0E40-9862-B8308F8A8DD8}"/>
+    <hyperlink ref="C11" r:id="rId2" xr:uid="{2ED25ACD-8A16-DD42-8FB2-9069856DDED4}"/>
+    <hyperlink ref="C12" r:id="rId3" xr:uid="{432655B1-7C28-0E40-9862-B8308F8A8DD8}"/>
     <hyperlink ref="C3" r:id="rId4" xr:uid="{A65943FD-A8AA-0141-8300-C953B43F032A}"/>
+    <hyperlink ref="C4" r:id="rId5" xr:uid="{5C5E8BDF-807F-974A-926D-5FE93B49A08D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>